<commit_message>
ETL Production 2007 - 2024
</commit_message>
<xml_diff>
--- a/reports/Fuentes de Información.xlsx
+++ b/reports/Fuentes de Información.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\ddayann\proyectos\Coffe\proyecto_aplicado_en_analitica_de_datos\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22E2AD37-4D08-44EF-A9D3-8D2463100312}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF6FD5DE-4C6A-48C9-B784-5B6787DAC86B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19110" yWindow="0" windowWidth="19380" windowHeight="20970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="19380" windowHeight="20970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="21">
   <si>
     <t>Variable</t>
   </si>
@@ -79,6 +79,15 @@
   </si>
   <si>
     <t>Anual</t>
+  </si>
+  <si>
+    <t>DAC</t>
+  </si>
+  <si>
+    <t>https://www.datos.gov.co/Agricultura-y-Desarrollo-Rural/Evaluaciones-Agropecuarias-Municipales-EVA/2pnw-mmge/about_data</t>
+  </si>
+  <si>
+    <t>Evaluaciones_Agropecuarias_Municipales_EVA_20260423.csv</t>
   </si>
 </sst>
 </file>
@@ -153,8 +162,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4D4160E0-7549-4F7A-B79F-A83FBBAED420}" name="Table1" displayName="Table1" ref="A1:H3" totalsRowShown="0">
-  <autoFilter ref="A1:H3" xr:uid="{4D4160E0-7549-4F7A-B79F-A83FBBAED420}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4D4160E0-7549-4F7A-B79F-A83FBBAED420}" name="Table1" displayName="Table1" ref="A1:H4" totalsRowShown="0">
+  <autoFilter ref="A1:H4" xr:uid="{4D4160E0-7549-4F7A-B79F-A83FBBAED420}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{CABC37A0-5FF1-4CC8-A13F-9835C1D33CE1}" name="Variable"/>
     <tableColumn id="2" xr3:uid="{161B5EA8-C96F-4F82-8C1A-D5A4E976E60B}" name="Entidad"/>
@@ -432,7 +441,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.08984375" bestFit="1" customWidth="1"/>
@@ -523,14 +532,41 @@
         <v>17</v>
       </c>
     </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="1">
+        <v>39083</v>
+      </c>
+      <c r="E4" s="1">
+        <v>43465</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H4" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1" xr:uid="{120242BE-B1FC-4797-AAA7-A16FEB24559C}"/>
     <hyperlink ref="F3" r:id="rId2" xr:uid="{7C7F8B47-00C7-4138-BA05-3A5691129DEB}"/>
+    <hyperlink ref="F4" r:id="rId3" xr:uid="{EA31A003-8EFF-41CB-97CC-C58FD33C8922}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ajuste DB Municipios para ee
</commit_message>
<xml_diff>
--- a/reports/Fuentes de Información.xlsx
+++ b/reports/Fuentes de Información.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\ddayann\proyectos\Coffe\proyecto_aplicado_en_analitica_de_datos\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF6FD5DE-4C6A-48C9-B784-5B6787DAC86B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6C6F901-DD81-4953-86AC-9F12357DF9A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="19380" windowHeight="20970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="18570" yWindow="3800" windowWidth="16570" windowHeight="16210" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,8 +24,31 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Dayan</author>
+  </authors>
+  <commentList>
+    <comment ref="G5" authorId="0" shapeId="0" xr:uid="{CB20BDD5-D8C0-4D7C-BBDD-7C94BECF19A2}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>https://www.colombiaenmapas.gov.co/?e=-94.63816516601295,-20.145273689787064,-53.856915166023796,29.452421339221825,4686&amp;b=igac&amp;u=0&amp;t=29&amp;servicio=610</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="26">
   <si>
     <t>Variable</t>
   </si>
@@ -88,13 +111,28 @@
   </si>
   <si>
     <t>Evaluaciones_Agropecuarias_Municipales_EVA_20260423.csv</t>
+  </si>
+  <si>
+    <t>Municipios</t>
+  </si>
+  <si>
+    <t>IGAC</t>
+  </si>
+  <si>
+    <t>Municipios, Distritos y Áreas no municipalizadas de Colombia</t>
+  </si>
+  <si>
+    <t>General</t>
+  </si>
+  <si>
+    <t>https://www.colombiaenmapas.gov.co/#</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -109,6 +147,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -162,8 +206,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4D4160E0-7549-4F7A-B79F-A83FBBAED420}" name="Table1" displayName="Table1" ref="A1:H4" totalsRowShown="0">
-  <autoFilter ref="A1:H4" xr:uid="{4D4160E0-7549-4F7A-B79F-A83FBBAED420}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4D4160E0-7549-4F7A-B79F-A83FBBAED420}" name="Table1" displayName="Table1" ref="A1:H5" totalsRowShown="0">
+  <autoFilter ref="A1:H5" xr:uid="{4D4160E0-7549-4F7A-B79F-A83FBBAED420}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{CABC37A0-5FF1-4CC8-A13F-9835C1D33CE1}" name="Variable"/>
     <tableColumn id="2" xr3:uid="{161B5EA8-C96F-4F82-8C1A-D5A4E976E60B}" name="Entidad"/>
@@ -440,14 +484,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.08984375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.26953125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.6328125" customWidth="1"/>
-    <col min="4" max="4" width="8.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.453125" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.6328125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.6328125" customWidth="1"/>
     <col min="7" max="7" width="50.7265625" bestFit="1" customWidth="1"/>
@@ -558,6 +602,32 @@
         <v>17</v>
       </c>
     </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="1">
+        <v>45658</v>
+      </c>
+      <c r="E5" s="1">
+        <v>46022</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" t="s">
+        <v>23</v>
+      </c>
+      <c r="H5" t="s">
+        <v>24</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1" xr:uid="{120242BE-B1FC-4797-AAA7-A16FEB24559C}"/>
@@ -565,8 +635,9 @@
     <hyperlink ref="F4" r:id="rId3" xr:uid="{EA31A003-8EFF-41CB-97CC-C58FD33C8922}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId4"/>
   <tableParts count="1">
-    <tablePart r:id="rId4"/>
+    <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
evapotransporación - mensual & anual 2005 - 2025
</commit_message>
<xml_diff>
--- a/reports/Fuentes de Información.xlsx
+++ b/reports/Fuentes de Información.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\ddayann\proyectos\Coffe\proyecto_aplicado_en_analitica_de_datos\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6C6F901-DD81-4953-86AC-9F12357DF9A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2469DF9C-9814-4854-838D-7304AC074958}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18570" yWindow="3800" windowWidth="16570" windowHeight="16210" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28710" yWindow="8090" windowWidth="9780" windowHeight="12880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="41">
   <si>
     <t>Variable</t>
   </si>
@@ -126,6 +126,51 @@
   </si>
   <si>
     <t>https://www.colombiaenmapas.gov.co/#</t>
+  </si>
+  <si>
+    <t>NDVI</t>
+  </si>
+  <si>
+    <t>Google</t>
+  </si>
+  <si>
+    <t>MODIS/061/MOD13Q1</t>
+  </si>
+  <si>
+    <t>https://code.earthengine.google.com/'ee-cafe-494102'</t>
+  </si>
+  <si>
+    <t>ndvi_municipal_mod13q1_2005_2025.csv</t>
+  </si>
+  <si>
+    <t>Diaria</t>
+  </si>
+  <si>
+    <t>Precipitación</t>
+  </si>
+  <si>
+    <t>Temperatura</t>
+  </si>
+  <si>
+    <t>Evapotranspiración</t>
+  </si>
+  <si>
+    <t>UCSB-CHG/CHIRPS/DAILY</t>
+  </si>
+  <si>
+    <t>precipitacion_municipal_chirps_2005_2025.csv</t>
+  </si>
+  <si>
+    <t>ECMWF/ERA5_LAND/DAILY_AGGR</t>
+  </si>
+  <si>
+    <t>temperatura_municipal_era5_2005_2025.csv</t>
+  </si>
+  <si>
+    <t>IDAHO_EPSCOR/TERRACLIMATE</t>
+  </si>
+  <si>
+    <t>evapotranspiracion_municipal_terraclimate_2005_2025.csv</t>
   </si>
 </sst>
 </file>
@@ -206,8 +251,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4D4160E0-7549-4F7A-B79F-A83FBBAED420}" name="Table1" displayName="Table1" ref="A1:H5" totalsRowShown="0">
-  <autoFilter ref="A1:H5" xr:uid="{4D4160E0-7549-4F7A-B79F-A83FBBAED420}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4D4160E0-7549-4F7A-B79F-A83FBBAED420}" name="Table1" displayName="Table1" ref="A1:H9" totalsRowShown="0">
+  <autoFilter ref="A1:H9" xr:uid="{4D4160E0-7549-4F7A-B79F-A83FBBAED420}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{CABC37A0-5FF1-4CC8-A13F-9835C1D33CE1}" name="Variable"/>
     <tableColumn id="2" xr3:uid="{161B5EA8-C96F-4F82-8C1A-D5A4E976E60B}" name="Entidad"/>
@@ -485,12 +530,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.08984375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.6328125" customWidth="1"/>
+    <col min="3" max="3" width="28.08984375" customWidth="1"/>
     <col min="4" max="4" width="9.453125" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.6328125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.6328125" customWidth="1"/>
@@ -628,16 +673,124 @@
         <v>24</v>
       </c>
     </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="1">
+        <v>45658</v>
+      </c>
+      <c r="E6" s="1">
+        <v>46022</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G6" t="s">
+        <v>30</v>
+      </c>
+      <c r="H6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" s="1">
+        <v>45658</v>
+      </c>
+      <c r="E7" s="1">
+        <v>46022</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G7" t="s">
+        <v>36</v>
+      </c>
+      <c r="H7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" s="1">
+        <v>45658</v>
+      </c>
+      <c r="E8" s="1">
+        <v>46022</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G8" t="s">
+        <v>38</v>
+      </c>
+      <c r="H8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" t="s">
+        <v>39</v>
+      </c>
+      <c r="D9" s="1">
+        <v>45658</v>
+      </c>
+      <c r="E9" s="1">
+        <v>46022</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G9" t="s">
+        <v>40</v>
+      </c>
+      <c r="H9" t="s">
+        <v>31</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1" xr:uid="{120242BE-B1FC-4797-AAA7-A16FEB24559C}"/>
     <hyperlink ref="F3" r:id="rId2" xr:uid="{7C7F8B47-00C7-4138-BA05-3A5691129DEB}"/>
     <hyperlink ref="F4" r:id="rId3" xr:uid="{EA31A003-8EFF-41CB-97CC-C58FD33C8922}"/>
+    <hyperlink ref="F6" r:id="rId4" xr:uid="{CFFEE9D5-04C7-42A1-8E3B-845255C9797C}"/>
+    <hyperlink ref="F7" r:id="rId5" xr:uid="{8E6A1BEF-EB60-43D2-B988-1CEA671BEFDC}"/>
+    <hyperlink ref="F8" r:id="rId6" xr:uid="{14B74280-392A-4DE7-9446-15B95E0EECFB}"/>
+    <hyperlink ref="F9" r:id="rId7" xr:uid="{2005D8BC-7DFA-425E-8311-C42D23C1D474}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId4"/>
+  <legacyDrawing r:id="rId8"/>
   <tableParts count="1">
-    <tablePart r:id="rId5"/>
+    <tablePart r:id="rId9"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>